<commit_message>
feat: close phase 1 contamination v1 and schema v1.1
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Canonical_Schema.xlsx
+++ b/NewLogic 03.05.2026/ST_Canonical_Schema.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="0_Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1_Sides" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2_Roles" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="3_EvidenceType" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="4_KnowledgeLevel" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="5_Confidence" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="6_ReliabilityFlags" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="7_Answer_Record" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="8_Respondent_Record" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="9_EvidenceItem_Record" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="10_AnalystAssessment" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="11_Contradiction_Record" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="12_RiskOutput_Record" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="13_RiskCategories" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="14_RoleCoverageMatrix" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="15_ConfidenceGate" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="16_OverridePrecedence" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="17_AnalystGate" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="18_VisualStandard" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="19_ChangeLog" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0_Index" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1_Sides" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2_Roles" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_EvidenceType" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_KnowledgeLevel" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Confidence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_ReliabilityFlags" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Answer_Record" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8_Respondent_Record" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9_EvidenceItem_Record" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_AnalystAssessment" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Contradiction_Record" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_RiskOutput_Record" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_RiskCategories" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_RoleCoverageMatrix" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_ConfidenceGate" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16_OverridePrecedence" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_AnalystGate" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18_VisualStandard" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19_ChangeLog" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -512,7 +512,7 @@
     <row r="1" ht="30" customHeight="1" s="13">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>STRUCTURAL TYPOLOGY · CANONICAL SCHEMA · v1.0</t>
+          <t>STRUCTURAL TYPOLOGY · CANONICAL SCHEMA · v1.1</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Nine flags identifying answer-reliability concerns</t>
+          <t>Ten flags identifying answer-reliability concerns</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
@@ -4171,7 +4171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="12" min="1" max="1"/>
@@ -4228,6 +4228,28 @@
       <c r="D3" s="23" t="inlineStr">
         <is>
           <t>Initial canonical schema. Resolves architectural critique that respondent answers were treated as truth. Adds 6 enums, 6 record types, 4 rule sheets, role coverage matrix, confidence gate, override precedence, analyst gate. Foundation for the 2026-05-03 rebuild brief.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1" s="13">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>Nikolai Petyaev (methodology decision)</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Adds tenth AnswerReliabilityFlag acquisition_framing_contamination (target-side only; excluded from primary score; retained as divergence record) — legislates the TSAM v3.1 / EDv2 v3.1 target-specific extension. Adds 8_Respondent_Record.acquisitionAwareness (conditional, target side).</t>
         </is>
       </c>
     </row>
@@ -5470,7 +5492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="36" customWidth="1" style="12" min="1" max="1"/>
@@ -5710,6 +5732,28 @@
       <c r="D12" s="21" t="inlineStr">
         <is>
           <t>Answer excluded from primary score; preserved for coverage map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1" s="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>acquisition_framing_contamination</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Acquisition-framing contamination</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Target-side respondent (Respondent.side = target) is aware of the pending acquisition (acquisitionAwareness = yes); the deal context may be colouring the answer toward acceptability or self-protection. Self-declarable by the respondent on any answer; mandatory on every answer when observationTenureMonths &lt; 18 or the respondent is in active acquisition discussions.</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>Answer excluded from primary score; retained as a divergence record against acquirer-observer evidence and surfaced for mandatory analyst review.</t>
         </is>
       </c>
     </row>
@@ -6273,7 +6317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="12" min="1" max="1"/>
@@ -6594,55 +6638,82 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="13">
+    <row r="14" ht="65" customHeight="1" s="13">
       <c r="A14" s="20" t="inlineStr">
         <is>
+          <t>acquisitionAwareness</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>enum: yes / no / partial</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>Conditional — required when side = target; null otherwise</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>Awareness of the pending acquisition. yes → engine sets respondent-level contamination signal and publishes it as a contamination indicator (TSAM 6 r7). partial → stored, does not trigger the signal. Domain alias: "deal awareness" (Triage 3 r6).</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="13">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
           <t>createdAt</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B15" s="23" t="inlineStr">
         <is>
           <t>ISO 8601 datetime</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D15" s="23" t="inlineStr">
         <is>
           <t>Server-side timestamp of profile creation.</t>
         </is>
       </c>
-      <c r="E14" s="21" t="inlineStr">
+      <c r="E15" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="23.85" customHeight="1" s="13">
-      <c r="A15" s="22" t="inlineStr">
+    <row r="16" ht="23.85" customHeight="1" s="13">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>analystVerified</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="D15" s="23" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Has the analyst reviewed and verified this respondent's role and access scope.</t>
         </is>
       </c>
-      <c r="E15" s="23" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>10_AnalystAssessment</t>
         </is>

</xml_diff>

<commit_message>
fix: align canonical schema with observation scope
</commit_message>
<xml_diff>
--- a/NewLogic 03.05.2026/ST_Canonical_Schema.xlsx
+++ b/NewLogic 03.05.2026/ST_Canonical_Schema.xlsx
@@ -512,7 +512,7 @@
     <row r="1" ht="30" customHeight="1" s="13">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>STRUCTURAL TYPOLOGY · CANONICAL SCHEMA · v1.1</t>
+          <t>STRUCTURAL TYPOLOGY · CANONICAL SCHEMA · v1.2</t>
         </is>
       </c>
     </row>
@@ -3381,14 +3381,14 @@
     <row r="1" ht="30" customHeight="1" s="13">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>OVERRIDE PRECEDENCE · target self-assessment vs target-observer scoring</t>
+          <t>OVERRIDE PRECEDENCE · target self-assessment vs target observer / inter-side precedence. This sheet governs target self-assessment vs target observer / inter-side precedence. It is not a universal evidence hierarchy.</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="13">
       <c r="A2" s="24" t="inlineStr">
         <is>
-          <t>PROVISIONAL DEFAULT (Q4). Resolves a structural ambiguity present in the prior architecture: whose answer wins when target self-assessment and acquirer-observed answers disagree.</t>
+          <t>PROVISIONAL DEFAULT (Q4). Resolves a structural ambiguity present in the prior architecture: whose answer wins when target self-assessment and acquirer-observed answers disagree. No universal document &gt; human rule exists outside this stated inter-side domain. Same-side Dual corroboration is outside the scope of this sheet. Accepted same-side Dual factors remain independence, diagnostic relevance, actual-event linkage, resistance to strategic tailoring, and provenance; they are not numerically ranked here.</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3456,7 @@
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>Document trumps self-report.</t>
+          <t>Within this inter-side target-self-vs-observer precedence domain only: documentary evidence governs over target self-report. Not a universal document&gt;human rule. Same-side Dual corroboration is outside this sheet.</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Document trumps observer claim.</t>
+          <t>Within this inter-side target-self-vs-observer precedence domain only: documentary evidence governs over the observer claim. Not a universal document&gt;human rule. Same-side Dual corroboration is outside this sheet.</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="12" min="1" max="1"/>
@@ -4250,6 +4250,28 @@
       <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Adds tenth AnswerReliabilityFlag acquisition_framing_contamination (target-side only; excluded from primary score; retained as divergence record) — legislates the TSAM v3.1 / EDv2 v3.1 target-specific extension. Adds 8_Respondent_Record.acquisitionAwareness (conditional, target side).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="20" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>Owner-authorized X-3 Canonical Schema correction</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>S-1 domain split for speaks_for_group_without_access (Dual AEM/TSAM Q1–Q11 → Dual 11_Role_Question_Scope; deal/workstream → 2_Roles; no bare-Q mapping). S-2 causal dedup: same access/scope cause must not force evidenceType = inference or add a second reliability/quality penalty. S-3 overgeneralized requires independent extrapolation evidence; scope mismatch alone insufficient; 0.5 unchanged. S-4 seniority mapping referenced to Dual sheet 11; no duplicated mapping; no new seniorityTier field. S-5 accessLevel clarified as routing/review/anomaly metadata only, not UseClass/cap/multiplier. S-6 namespaced question identity: persisted Answer.questionId = globally namespaced Question.id; bare Q1 prohibited as a global ID. S-8 unspecified → UNRESOLVED → practitioner review; no fallback. S-9 inter-side precedence scope; no universal document&gt;human. X-3 CORR1 inference-layer boundary: evidenceType = inference does not by itself lower Observation Use Class or imply access failure. S-7: no new universal formula encoded.</t>
         </is>
       </c>
     </row>
@@ -4878,7 +4900,7 @@
       </c>
       <c r="D24" s="21" t="inlineStr">
         <is>
-          <t>Requires free-text role description and analyst review for access scoping</t>
+          <t>Requires free-text role description and analyst review for access scoping. Dual AEM/TSAM Q1–Q11 compatibility: roleCode = unspecified → UNRESOLVED → practitioner access review. No fallback tier. No conversion to external. No conversion to line_level. No default PRIMARY. No default CONTEXTUAL. No multiplier substitution. The five-state comparator must not proceed until review.</t>
         </is>
       </c>
       <c r="E24" s="21" t="inlineStr">
@@ -5638,12 +5660,12 @@
       </c>
       <c r="C8" s="21" t="inlineStr">
         <is>
-          <t>Respondent answered for the entire organisation when their access scope is narrower.</t>
+          <t>Content-level extrapolation beyond actual evidence. Scope mismatch or observation-altitude mismatch alone is insufficient. Allowed only when there is independent evidence that the respondent extrapolates beyond observed events, observed roles, observed functions, observed time period, or an otherwise supported evidence base.</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Answer downweighted by 0.5; flagged for role-mismatch review.</t>
+          <t>Answer downweighted by 0.5; flagged for role-mismatch review. If the same underlying access/scope cause is already adjudicated through Observation Use Class or speaks_for_group_without_access, do not apply an additional overgeneralized penalty unless separate extrapolation evidence exists.</t>
         </is>
       </c>
     </row>
@@ -5660,12 +5682,12 @@
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Respondent answered a question outside their legitimate access map (Sheet 2_Roles).</t>
+          <t>Domain split. For AEM Q1–Q11 and TSAM Q1–Q11, legitimate observation access is determined by ST_Dual_Respondent_Axis_Comparison_v1.xlsx sheet 11_Role_Question_Scope using accepted Observation Scope logic. Bare local IDs such as Q1 must not be mapped to Dual from other instruments. For deal/workstream questions, sheet 2_Roles remains the authority for its original deal/workstream legitimate-access domain. For EDv2 or other instruments, Dual access logic must not be applied from bare Q1…Qn; only instrument-specific authority may be used. Missing instrument-specific authority is not invented here.</t>
         </is>
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Answer scored as inference at most, regardless of self-reported EvidenceType.</t>
+          <t>Audit/reliability marker. If the same access/scope cause has already changed Observation Use Class: do NOT force evidenceType = inference; do NOT apply an additional reliability downweight for that same cause; do NOT create another independent evidence-quality penalty. evidenceType = inference may be assigned only when independently supported by the answer's actual evidentiary basis; this flag does not automatically force evidenceType = inference. In legacy deal/workstream contexts without Observation Use Class, the existing access effect may remain the single applicable legacy effect, but the same flag must not be counted twice. Numeric evidence weights are unchanged.</t>
         </is>
       </c>
     </row>
@@ -5897,12 +5919,12 @@
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Stable identifier of the question, e.g. ACQ-Q1, TGT-OBS-Q5.</t>
+          <t>Persisted Answer.questionId must equal the globally namespaced stable Question.id. Bare local IDs such as Q1, Q2 must NOT be persisted as globally unique identifiers. Field name unchanged.</t>
         </is>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>See per-questionnaire keys</t>
+          <t>Question resolution is questionnaire/instrument namespaced. Safe logical key: (moduleId, workbookQuestionId). Physical source equivalent: (sourceWorkbook, sourceSheet, workbookQuestionId). Dual local questionRef may only be resolved after confirming the instrument/module. Authorized Dual mapping: (acquirerEnvironment, Q1…Q11) → Dual Q1…Q11; (targetSelfAssessment, Q1…Q11) → Dual Q1…Q11. Prohibited: bare Q1 → Dual Q1; environmentLevel1 Q1 → Dual Q1. Existing IDs are not renamed.</t>
         </is>
       </c>
     </row>
@@ -6521,12 +6543,12 @@
       </c>
       <c r="D9" s="23" t="inlineStr">
         <is>
-          <t>Decision authority and observation altitude.</t>
+          <t>Decision authority and observation altitude. For Dual AEM/TSAM Observation Scope, seniority tier mapping is owned by ST_Dual_Respondent_Axis_Comparison_v1.xlsx sheet 11_Role_Question_Scope. Canonical Schema does not duplicate that mapping and does not add a seniorityTier field.</t>
         </is>
       </c>
       <c r="E9" s="23" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ST_Dual_Respondent_Axis_Comparison_v1.xlsx · 11_Role_Question_Scope · Seniority Tier Mapping</t>
         </is>
       </c>
     </row>
@@ -6548,7 +6570,7 @@
       </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
-          <t>Scope of legitimate organisational visibility.</t>
+          <t>Respondent-wide visibility metadata for routing, practitioner review, and anomaly detection. Must NOT by itself determine question-level Observation Use Class, cap question-level Observation Use Class, modify Evidence Quality, or act as a multiplier. Question-level actual access is established through applicable Observation Scope rules, per-answer directObservationGate, and question-qualified option semantics where relevant. Enum remains full | functional | limited | external_only.</t>
         </is>
       </c>
       <c r="E10" s="21" t="inlineStr">

</xml_diff>